<commit_message>
Switch from pain records to products (ProductsDb.dbo.Products)
- New products.js data layer for Id, Name, Price decimal(10,2), Stock, ImageUrl;
  validation matches the column types, accepts "$1,299.50" style prices and
  flexible headers (ImageUrl / Image URL / image_url)
- Hard delete, since the table has no soft-delete column
- AI extractor now reads products from supplier emails (unit price, stock,
  image link; missing values are flagged, never guessed)
- REST API moved to /api/products; web app shows thumbnails and stock badges
- Product sample attachments, Gmail label products-processed, README rewritten

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/samples/data1-sample.xlsx
+++ b/server/samples/data1-sample.xlsx
@@ -4,64 +4,40 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="PainRecords" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Products" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>patient_name</t>
-  </si>
-  <si>
-    <t>country</t>
-  </si>
-  <si>
-    <t>pain_level</t>
-  </si>
-  <si>
-    <t>pain_location</t>
-  </si>
-  <si>
-    <t>occurred_at</t>
-  </si>
-  <si>
-    <t>notes</t>
-  </si>
-  <si>
-    <t>Email Test One</t>
-  </si>
-  <si>
-    <t>India</t>
-  </si>
-  <si>
-    <t>Lower back</t>
-  </si>
-  <si>
-    <t>Imported from Excel</t>
-  </si>
-  <si>
-    <t>Email Test Two</t>
-  </si>
-  <si>
-    <t>Canada</t>
-  </si>
-  <si>
-    <t>Wrist</t>
-  </si>
-  <si>
-    <t/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Stock</t>
+  </si>
+  <si>
+    <t>ImageUrl</t>
+  </si>
+  <si>
+    <t>Wireless Mouse - Black</t>
+  </si>
+  <si>
+    <t>https://example.com/images/mouse-black.jpg</t>
+  </si>
+  <si>
+    <t>USB-C Charging Cable 2m</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm"/>
-  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -96,9 +72,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -438,22 +414,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="11" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="20" style="1" customWidth="1"/>
-    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="10" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -462,51 +436,30 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="B2" s="1">
+        <v>24.99</v>
+      </c>
+      <c r="C2">
+        <v>120</v>
+      </c>
+      <c r="D2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="1">
-        <v>46294.05208333333</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
+      <c r="B3" s="1">
+        <v>9.5</v>
       </c>
       <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="1">
-        <v>46295.25</v>
-      </c>
-      <c r="F3" t="s">
-        <v>13</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>